<commit_message>
L5: add model-detail reference data + source pointers; L9: fix starter=solution on incident sheets
L5 (AI Model Governance): add exercises/starter/data/ — per-model fact sheets
(M001/M002/M006) and model_details_reference.md — so students work from given
facts instead of inventing values. Notebook Part 1/Part 5 markdown and README
point to data/; code cells unchanged.

L9 (AI Incident Management): replace starter with corrected version — Incident
Playbook and Severity Classification were identical to the solution; now blanked
for genuine student work (all 4 sheets have real gaps).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lesson-9-ai-incident-management/exercises/starter/incident_response_starter.xlsx
+++ b/lesson-9-ai-incident-management/exercises/starter/incident_response_starter.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,8 +49,18 @@
       <b val="1"/>
       <color rgb="00000000"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="FF888888"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="FF888888"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -117,6 +127,16 @@
         <bgColor rgb="00FFB6C1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4EC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -136,7 +156,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -179,6 +199,22 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -544,7 +580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -676,6 +712,37 @@
       <c r="A17" s="5" t="inlineStr">
         <is>
           <t>• Must report certain incidents to NTSB and FTA within mandated timeframes</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>COLOR LEGEND:</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>Pre-filled</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Context provided — do not change.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>Your work</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Cells marked TO BE FILLED — replace with your answer. Gray hints are prompts, not answers.</t>
         </is>
       </c>
     </row>
@@ -795,37 +862,37 @@
           <t>Routes through certain neighborhoods receive longer travel times</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="E2" s="22" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="F2" s="22" t="inlineStr">
         <is>
           <t>Monitor route fairness metrics across regions; compare avg travel times</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="G2" s="22" t="inlineStr">
         <is>
           <t>Pause affected routes; escalate to ML team; notify operations</t>
         </is>
       </c>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="H2" s="22" t="inlineStr">
         <is>
           <t>Review training data distribution; analyze prediction patterns by geography</t>
         </is>
       </c>
-      <c r="I2" s="7" t="inlineStr">
+      <c r="I2" s="22" t="inlineStr">
         <is>
           <t>Retrain with balanced data; implement fairness constraints; add monitoring</t>
         </is>
       </c>
-      <c r="J2" s="7" t="inlineStr">
+      <c r="J2" s="22" t="inlineStr">
         <is>
           <t>Notify affected route managers; customer support alert</t>
         </is>
       </c>
-      <c r="K2" s="7" t="inlineStr">
+      <c r="K2" s="22" t="inlineStr">
         <is>
           <t>Document root cause; update training pipeline; implement fairness dashboard</t>
         </is>
@@ -852,37 +919,37 @@
           <t>Chatbot provides rude or discriminatory responses to passenger inquiries</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="22" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="F3" s="22" t="inlineStr">
         <is>
           <t>Content filtering; customer complaints; automated toxicity detection</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="G3" s="22" t="inlineStr">
         <is>
           <t>Disable chatbot; escalate to content team; begin log analysis</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="H3" s="22" t="inlineStr">
         <is>
           <t>Review chat logs; identify trigger phrases; check outputs for toxicity</t>
         </is>
       </c>
-      <c r="I3" s="7" t="inlineStr">
+      <c r="I3" s="22" t="inlineStr">
         <is>
           <t>Apply content filters; retrain with safer examples; add guardrails</t>
         </is>
       </c>
-      <c r="J3" s="7" t="inlineStr">
+      <c r="J3" s="22" t="inlineStr">
         <is>
           <t>Apologize to passengers; notify customer service teams</t>
         </is>
       </c>
-      <c r="K3" s="7" t="inlineStr">
+      <c r="K3" s="22" t="inlineStr">
         <is>
           <t>Update chatbot guidelines; implement content moderation</t>
         </is>
@@ -909,39 +976,44 @@
           <t>Route accuracy drops from 94% to 78% during morning rush</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>Monitor accuracy and latency with time-based thresholds</t>
-        </is>
-      </c>
-      <c r="G4" s="7" t="inlineStr">
-        <is>
-          <t>Scale infrastructure; enable fallback models; notify passengers</t>
-        </is>
-      </c>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
-          <t>Analyze resource usage; profile model inference time</t>
-        </is>
-      </c>
-      <c r="I4" s="7" t="inlineStr">
-        <is>
-          <t>Optimize inference; add compute capacity; implement caching</t>
-        </is>
-      </c>
-      <c r="J4" s="7" t="inlineStr">
-        <is>
-          <t>Service degradation notice; daily updates to operations</t>
-        </is>
-      </c>
-      <c r="K4" s="7" t="inlineStr">
-        <is>
-          <t>Implement load testing; establish baseline SLAs</t>
+      <c r="E4" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(which severity? S1–S4)</t>
+        </is>
+      </c>
+      <c r="F4" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(how would you catch it?)</t>
+        </is>
+      </c>
+      <c r="G4" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(first-hour containment?)</t>
+        </is>
+      </c>
+      <c r="H4" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED</t>
+        </is>
+      </c>
+      <c r="I4" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED</t>
+        </is>
+      </c>
+      <c r="J4" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(who needs to know?)</t>
+        </is>
+      </c>
+      <c r="K4" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(prevent recurrence?)</t>
         </is>
       </c>
     </row>
@@ -966,39 +1038,44 @@
           <t>Personal location data and payment info exposed via API vulnerability</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>S1</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>Security monitoring; audit logs; anomalous API access patterns</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
-        <is>
-          <t>Take system offline; activate incident response team; preserve evidence</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>Forensic analysis; determine scope of exposure; identify affected users</t>
-        </is>
-      </c>
-      <c r="I5" s="7" t="inlineStr">
-        <is>
-          <t>Patch vulnerability; rotate credentials; implement encryption</t>
-        </is>
-      </c>
-      <c r="J5" s="7" t="inlineStr">
-        <is>
-          <t>Notify legal; customer notification per regulations; regulator reporting</t>
-        </is>
-      </c>
-      <c r="K5" s="7" t="inlineStr">
-        <is>
-          <t>Offer credit monitoring; security audit; improve access controls</t>
+      <c r="E5" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(which severity? S1–S4)</t>
+        </is>
+      </c>
+      <c r="F5" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(how would you catch it?)</t>
+        </is>
+      </c>
+      <c r="G5" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(first-hour containment?)</t>
+        </is>
+      </c>
+      <c r="H5" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED</t>
+        </is>
+      </c>
+      <c r="I5" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED</t>
+        </is>
+      </c>
+      <c r="J5" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(who needs to know?)</t>
+        </is>
+      </c>
+      <c r="K5" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(prevent recurrence?)</t>
         </is>
       </c>
     </row>
@@ -1023,39 +1100,44 @@
           <t>Route guidance includes non-existent roads or omits safety warnings</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>S1</t>
-        </is>
-      </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>User feedback; verification against actual road data; safety audits</t>
-        </is>
-      </c>
-      <c r="G6" s="7" t="inlineStr">
-        <is>
-          <t>Issue safety alert; disable affected guidance; activate crisis team</t>
-        </is>
-      </c>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>Review hallucination patterns; check training data for errors</t>
-        </is>
-      </c>
-      <c r="I6" s="7" t="inlineStr">
-        <is>
-          <t>Implement hallucination detection; add fact-checking layer; retrain</t>
-        </is>
-      </c>
-      <c r="J6" s="7" t="inlineStr">
-        <is>
-          <t>Safety alert to all users; regulatory notifications; media statement</t>
-        </is>
-      </c>
-      <c r="K6" s="7" t="inlineStr">
-        <is>
-          <t>Establish ground truth verification; add confidence scoring</t>
+      <c r="E6" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(which severity? S1–S4)</t>
+        </is>
+      </c>
+      <c r="F6" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(how would you catch it?)</t>
+        </is>
+      </c>
+      <c r="G6" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(first-hour containment?)</t>
+        </is>
+      </c>
+      <c r="H6" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED</t>
+        </is>
+      </c>
+      <c r="I6" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED</t>
+        </is>
+      </c>
+      <c r="J6" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(who needs to know?)</t>
+        </is>
+      </c>
+      <c r="K6" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(prevent recurrence?)</t>
         </is>
       </c>
     </row>
@@ -1080,39 +1162,44 @@
           <t>Kubernetes cluster crash; database connection failure</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>S1</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>Health checks; availability monitoring; customer reports; error spikes</t>
-        </is>
-      </c>
-      <c r="G7" s="7" t="inlineStr">
-        <is>
-          <t>Activate incident commander; initiate failover; notify all stakeholders</t>
-        </is>
-      </c>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>Review deployment logs; analyze infrastructure metrics; check recent changes</t>
-        </is>
-      </c>
-      <c r="I7" s="7" t="inlineStr">
-        <is>
-          <t>Restore from backup; rollback deployment; fix infrastructure</t>
-        </is>
-      </c>
-      <c r="J7" s="7" t="inlineStr">
-        <is>
-          <t>Continuous status updates; customer notification; leadership briefing</t>
-        </is>
-      </c>
-      <c r="K7" s="7" t="inlineStr">
-        <is>
-          <t>Improve change management; add chaos engineering; improve monitoring</t>
+      <c r="E7" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(which severity? S1–S4)</t>
+        </is>
+      </c>
+      <c r="F7" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(how would you catch it?)</t>
+        </is>
+      </c>
+      <c r="G7" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(first-hour containment?)</t>
+        </is>
+      </c>
+      <c r="H7" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED</t>
+        </is>
+      </c>
+      <c r="I7" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED</t>
+        </is>
+      </c>
+      <c r="J7" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(who needs to know?)</t>
+        </is>
+      </c>
+      <c r="K7" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(prevent recurrence?)</t>
         </is>
       </c>
     </row>
@@ -1137,39 +1224,44 @@
           <t>Decisions made without explainability; violates data residency requirements</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>Compliance audits; regulatory reporting; legal review</t>
-        </is>
-      </c>
-      <c r="G8" s="7" t="inlineStr">
-        <is>
-          <t>Notify legal/compliance; suspend non-compliant features; prepare response</t>
-        </is>
-      </c>
-      <c r="H8" s="7" t="inlineStr">
-        <is>
-          <t>Audit compliance requirements; determine scope of violation</t>
-        </is>
-      </c>
-      <c r="I8" s="7" t="inlineStr">
-        <is>
-          <t>Implement required controls; add explainability; establish governance</t>
-        </is>
-      </c>
-      <c r="J8" s="7" t="inlineStr">
-        <is>
-          <t>Regulatory notification; legal coordination; customer transparency</t>
-        </is>
-      </c>
-      <c r="K8" s="7" t="inlineStr">
-        <is>
-          <t>Document compliance framework; implement continuous monitoring</t>
+      <c r="E8" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(which severity? S1–S4)</t>
+        </is>
+      </c>
+      <c r="F8" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(how would you catch it?)</t>
+        </is>
+      </c>
+      <c r="G8" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(first-hour containment?)</t>
+        </is>
+      </c>
+      <c r="H8" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED</t>
+        </is>
+      </c>
+      <c r="I8" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED</t>
+        </is>
+      </c>
+      <c r="J8" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(who needs to know?)</t>
+        </is>
+      </c>
+      <c r="K8" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(prevent recurrence?)</t>
         </is>
       </c>
     </row>
@@ -1194,46 +1286,44 @@
           <t>Coordinated requests with malicious patterns designed to degrade service</t>
         </is>
       </c>
-      <c r="E9" s="13" t="inlineStr">
-        <is>
-          <t>"S1"
-Reasoning: Deliberate manipulation of a safety-critical transit system poses immediate risk to passenger safety; classified as critical for rapid response.</t>
-        </is>
-      </c>
-      <c r="F9" s="13" t="inlineStr">
-        <is>
-          <t>"Anomaly detection algorithms, ML model behavior analysis, unusual request pattern analysis, behavioral fingerprinting"
-Reasoning: Combined detection methods help identify coordinated attack signatures across the system; behavioral analysis reveals non-organic request patterns.</t>
-        </is>
-      </c>
-      <c r="G9" s="13" t="inlineStr">
-        <is>
-          <t>"Rate limiting and request throttling; isolate affected routing service; notify security team; preserve logs for investigation"
-Reasoning: Immediate isolation prevents cascading failures; rate limiting stops attack propagation; preserving logs enables forensic analysis and attribution.</t>
-        </is>
-      </c>
-      <c r="H9" s="13" t="inlineStr">
-        <is>
-          <t>"Analyze attack patterns and signatures; determine scope of affected routes; assess whether passenger safety was compromised; review attacker capabilities"
-Reasoning: Pattern analysis identifies attack sophistication; scope assessment helps quantify impact; safety review ensures no undetected harm occurred.</t>
-        </is>
-      </c>
-      <c r="I9" s="13" t="inlineStr">
-        <is>
-          <t>"Implement input validation and adversarial robustness techniques; add intrusion detection; improve API authentication"
-Reasoning: Input validation blocks malformed requests; adversarial robustness hardens model; improved auth prevents credential-based attacks.</t>
-        </is>
-      </c>
-      <c r="J9" s="13" t="inlineStr">
-        <is>
-          <t>"Security alert to ops; law enforcement notification for potential coordinated attacks; briefing to executive team and board"
-Reasoning: Ops team needs immediate awareness; law enforcement may be necessary for prosecuting attackers; leadership needs to understand security posture impact.</t>
-        </is>
-      </c>
-      <c r="K9" s="13" t="inlineStr">
-        <is>
-          <t>"Adversarial testing against the routing engine; system hardening with cryptographic verification; threat modeling for supply chain attacks"
-Reasoning: Adversarial testing identifies similar vulnerabilities proactively; cryptographic verification prevents tampering; threat modeling improves long-term security posture.</t>
+      <c r="E9" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(which severity? S1–S4)</t>
+        </is>
+      </c>
+      <c r="F9" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(how would you catch it?)</t>
+        </is>
+      </c>
+      <c r="G9" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(first-hour containment?)</t>
+        </is>
+      </c>
+      <c r="H9" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED</t>
+        </is>
+      </c>
+      <c r="I9" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED</t>
+        </is>
+      </c>
+      <c r="J9" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(who needs to know?)</t>
+        </is>
+      </c>
+      <c r="K9" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(prevent recurrence?)</t>
         </is>
       </c>
     </row>
@@ -1258,46 +1348,44 @@
           <t>Historical route data tampered with to introduce systematic bias</t>
         </is>
       </c>
-      <c r="E10" s="13" t="inlineStr">
-        <is>
-          <t>"S1"
-Reasoning: Data poisoning undermines the integrity of all downstream models and decisions; threatens fundamental trust in the AI system.</t>
-        </is>
-      </c>
-      <c r="F10" s="13" t="inlineStr">
-        <is>
-          <t>"Data validation and statistical anomaly detection; performance baseline comparison; data lineage tracking; checksums on training data"
-Reasoning: Statistical anomalies reveal contamination; performance baselines show degradation; checksums and lineage enable identification of poisoned batches.</t>
-        </is>
-      </c>
-      <c r="G10" s="13" t="inlineStr">
-        <is>
-          <t>"Halt all retraining; isolate compromised data; preserve evidence chain; activate incident commander; notify Chief Data Officer"
-Reasoning: Stopping retraining prevents poisoned models from deployment; evidence preservation enables investigation; rapid escalation ensures proper oversight.</t>
-        </is>
-      </c>
-      <c r="H10" s="13" t="inlineStr">
-        <is>
-          <t>"Audit data pipeline end-to-end; identify contamination source and entry point; assess impact on existing trained models; review access logs"
-Reasoning: Pipeline audit reveals vulnerabilities; source identification prevents recurrence; impact assessment informs remediation scope; access logs identify insider threats.</t>
-        </is>
-      </c>
-      <c r="I10" s="13" t="inlineStr">
-        <is>
-          <t>"Data cleaning and validation; integrity checks at ingestion points; verified retraining with clean historical data; implement cryptographic integrity checks"
-Reasoning: Cleaning removes bad data; validation prevents future poisoning; verified retraining with curated data restores model trustworthiness; cryptographic checks ensure data hasn't been tampered.</t>
-        </is>
-      </c>
-      <c r="J10" s="13" t="inlineStr">
-        <is>
-          <t>"Data governance briefing to compliance and engineering; engineering team notification of process improvements; training for data handling"
-Reasoning: Governance needs awareness of vulnerabilities; engineering learns from incident; training prevents similar mistakes; transparency builds organizational resilience.</t>
-        </is>
-      </c>
-      <c r="K10" s="13" t="inlineStr">
-        <is>
-          <t>"Implement data validation gates in pipeline; fingerprinting of training data; stricter access controls; automated anomaly detection on data distributions"
-Reasoning: Validation gates catch issues early; fingerprinting enables quick identification; access controls limit poisoning opportunities; automated monitoring provides continuous safety.</t>
+      <c r="E10" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(which severity? S1–S4)</t>
+        </is>
+      </c>
+      <c r="F10" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(how would you catch it?)</t>
+        </is>
+      </c>
+      <c r="G10" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(first-hour containment?)</t>
+        </is>
+      </c>
+      <c r="H10" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED</t>
+        </is>
+      </c>
+      <c r="I10" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED</t>
+        </is>
+      </c>
+      <c r="J10" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(who needs to know?)</t>
+        </is>
+      </c>
+      <c r="K10" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(prevent recurrence?)</t>
         </is>
       </c>
     </row>
@@ -1322,46 +1410,44 @@
           <t>Former contractor retains access; API key exposed in public repository</t>
         </is>
       </c>
-      <c r="E11" s="13" t="inlineStr">
-        <is>
-          <t>"S1"
-Reasoning: Unauthorized access to an AI system controlling transit can enable data theft, system manipulation, or safety-critical routing errors affecting millions.</t>
-        </is>
-      </c>
-      <c r="F11" s="13" t="inlineStr">
-        <is>
-          <t>"Failed login attempts and rate limiting triggers; unusual access locations or times; off-hours access patterns; anomalous API key usage; geo-velocity checks"
-Reasoning: Failed attempts indicate compromise attempts; unusual patterns reveal unauthorized access; geo-velocity violations catch credential sharing; API anomalies show misuse.</t>
-        </is>
-      </c>
-      <c r="G11" s="13" t="inlineStr">
-        <is>
-          <t>"Immediate credential revocation; forced password reset for affected users; enable MFA across all accounts; revoke all API keys; disable compromised sessions"
-Reasoning: Revocation stops attackers immediately; forced resets prevent reuse; MFA makes future compromises harder; API key revocation blocks programmatic access; session termination logs out intruders.</t>
-        </is>
-      </c>
-      <c r="H11" s="13" t="inlineStr">
-        <is>
-          <t>"Comprehensive access log audit; determine scope of unauthorized actions; identify affected systems and data; assess attacker dwell time"
-Reasoning: Log audit reveals what attacker accessed; scope determines impact magnitude; dwell time assessment shows detection delay; comprehensive review prevents missing lateral movement.</t>
-        </is>
-      </c>
-      <c r="I11" s="13" t="inlineStr">
-        <is>
-          <t>"Stronger authentication (MFA/FIDO2); secret management and rotation; access review and removal of dormant accounts; hardware security keys for critical roles"
-Reasoning: MFA/FIDO2 prevents credential-based attacks; secret management prevents exposure; account cleanup reduces attack surface; hardware keys protect the highest-privilege accounts.</t>
-        </is>
-      </c>
-      <c r="J11" s="13" t="inlineStr">
-        <is>
-          <t>"Security briefing to all teams; notification to affected users; optional credit monitoring if personal data was accessed; regulatory notification if required"
-Reasoning: Team awareness improves future vigilance; user notification builds trust; credit monitoring addresses data breach concerns; regulatory notification meets compliance obligations.</t>
-        </is>
-      </c>
-      <c r="K11" s="13" t="inlineStr">
-        <is>
-          <t>"Credential rotation policy; enhanced audit logging; security awareness training; phishing simulations; regular access reviews"
-Reasoning: Regular rotation limits exposure window; audit logging improves detection; training reduces human vulnerabilities; simulations identify at-risk employees; reviews prevent privilege creep.</t>
+      <c r="E11" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(which severity? S1–S4)</t>
+        </is>
+      </c>
+      <c r="F11" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(how would you catch it?)</t>
+        </is>
+      </c>
+      <c r="G11" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(first-hour containment?)</t>
+        </is>
+      </c>
+      <c r="H11" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED</t>
+        </is>
+      </c>
+      <c r="I11" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED</t>
+        </is>
+      </c>
+      <c r="J11" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(who needs to know?)</t>
+        </is>
+      </c>
+      <c r="K11" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(prevent recurrence?)</t>
         </is>
       </c>
     </row>
@@ -1436,27 +1522,27 @@
           <t>S1</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" s="22" t="inlineStr">
         <is>
           <t>Immediate safety risk; potential data breach; system unavailable; passenger safety compromised</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="D2" s="22" t="inlineStr">
         <is>
           <t>&lt; 15 minutes</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="E2" s="22" t="inlineStr">
         <is>
           <t>CEO/Board; Legal; Chief Security Officer; NTSB/FTA</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="F2" s="22" t="inlineStr">
         <is>
           <t>All stakeholders; customers; regulators; media</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="G2" s="22" t="inlineStr">
         <is>
           <t>Data breach; System outage; Safety-critical hallucination</t>
         </is>
@@ -1473,29 +1559,33 @@
           <t>S2</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>Significant disruption; degraded experience; data integrity concerns; bias detected</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>&lt; 1 hour</t>
-        </is>
-      </c>
-      <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>VP Engineering; VP Product; Chief Compliance Officer</t>
-        </is>
-      </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>Leadership; affected customers; operations team</t>
-        </is>
-      </c>
-      <c r="G3" s="7" t="inlineStr">
-        <is>
-          <t>Model bias; Performance degradation; Chatbot issues; Adversarial attack</t>
+      <c r="C3" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(harm to whom?)</t>
+        </is>
+      </c>
+      <c r="D3" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(how fast?)</t>
+        </is>
+      </c>
+      <c r="E3" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(escalate to whom?)</t>
+        </is>
+      </c>
+      <c r="F3" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED</t>
+        </is>
+      </c>
+      <c r="G3" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(which incidents fit?)</t>
         </is>
       </c>
     </row>
@@ -1510,29 +1600,33 @@
           <t>S3</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>Degraded performance; workaround exists; limited passenger impact</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>&lt; 4 hours</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>Engineering Manager; Product Manager</t>
-        </is>
-      </c>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>Team leads; affected teams; management</t>
-        </is>
-      </c>
-      <c r="G4" s="7" t="inlineStr">
-        <is>
-          <t>Minor accuracy drop; Latency increase; Non-critical bug</t>
+      <c r="C4" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(harm to whom?)</t>
+        </is>
+      </c>
+      <c r="D4" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(how fast?)</t>
+        </is>
+      </c>
+      <c r="E4" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(escalate to whom?)</t>
+        </is>
+      </c>
+      <c r="F4" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED</t>
+        </is>
+      </c>
+      <c r="G4" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(which incidents fit?)</t>
         </is>
       </c>
     </row>
@@ -1547,29 +1641,33 @@
           <t>S4</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Minimal impact; cosmetic issue; isolated to small group</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>&lt; 24 hours</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>Team lead (no escalation)</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>Development team; knowledge base</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
-        <is>
-          <t>UI issue; Documentation error; Slow non-critical query</t>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(harm to whom?)</t>
+        </is>
+      </c>
+      <c r="D5" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(how fast?)</t>
+        </is>
+      </c>
+      <c r="E5" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(escalate to whom?)</t>
+        </is>
+      </c>
+      <c r="F5" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED</t>
+        </is>
+      </c>
+      <c r="G5" s="19" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(which incidents fit?)</t>
         </is>
       </c>
     </row>
@@ -1584,7 +1682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1634,399 +1732,414 @@
       </c>
     </row>
     <row r="2" ht="40" customHeight="1">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="22" t="inlineStr">
         <is>
           <t>1. Detection</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="B2" s="22" t="inlineStr">
         <is>
           <t>Identify anomaly through monitoring, alerts, or user reports</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" s="22" t="inlineStr">
         <is>
           <t>Monitoring System / Operations Team</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="D2" s="22" t="inlineStr">
         <is>
           <t>Real-time to 5 min</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="E2" s="22" t="inlineStr">
         <is>
           <t>Incident Alert Template</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="F2" s="22" t="inlineStr">
         <is>
           <t>Prometheus, DataDog, Support System</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="G2" s="22" t="inlineStr">
         <is>
           <t>Incident ticket created</t>
         </is>
       </c>
     </row>
     <row r="3" ht="40" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="22" t="inlineStr">
         <is>
           <t>2. Triage</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="22" t="inlineStr">
         <is>
           <t>Verify incident; assess immediate impact; gather initial context</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="22" t="inlineStr">
         <is>
           <t>On-Call Engineer / Incident Manager</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="22" t="inlineStr">
         <is>
           <t>5-15 minutes</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="22" t="inlineStr">
         <is>
           <t>Triage Assessment Form</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="F3" s="22" t="inlineStr">
         <is>
           <t>PagerDuty, Jira</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="G3" s="22" t="inlineStr">
         <is>
           <t>Confirmed incident with initial severity</t>
         </is>
       </c>
     </row>
     <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>3. Classification</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="22" t="inlineStr">
         <is>
           <t>Determine severity; assign category; set SLA response time</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>Incident Manager / Tech Lead</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>10-20 minutes</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>Classification Matrix</t>
-        </is>
-      </c>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>Incident Management Tool, Slack</t>
-        </is>
-      </c>
-      <c r="G4" s="7" t="inlineStr">
-        <is>
-          <t>Incident classified with severity and SLA</t>
+      <c r="C4" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(who owns this step?)</t>
+        </is>
+      </c>
+      <c r="D4" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(how fast?)</t>
+        </is>
+      </c>
+      <c r="E4" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(which template?)</t>
+        </is>
+      </c>
+      <c r="F4" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(which tools?)</t>
+        </is>
+      </c>
+      <c r="G4" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(what's produced?)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>4. Initial Response</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>Execute containment actions per playbook; engage necessary teams</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Engineering Lead / Operations</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>Within SLA</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>Incident Response Checklist</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>Runbooks, Slack, War Room</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
-        <is>
-          <t>Incident contained; teams engaged</t>
+      <c r="C5" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(who owns this step?)</t>
+        </is>
+      </c>
+      <c r="D5" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(how fast?)</t>
+        </is>
+      </c>
+      <c r="E5" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(which template?)</t>
+        </is>
+      </c>
+      <c r="F5" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(which tools?)</t>
+        </is>
+      </c>
+      <c r="G5" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(what's produced?)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>5. Investigation</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
         <is>
           <t>Detailed analysis; gather logs and metrics; identify root cause</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>Data Scientists / Engineers / Security</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>1-48 hours</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>Investigation Log Template</t>
-        </is>
-      </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>ELK Stack, Jupyter, Git</t>
-        </is>
-      </c>
-      <c r="G6" s="7" t="inlineStr">
-        <is>
-          <t>Root cause identified</t>
+      <c r="C6" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(who owns this step?)</t>
+        </is>
+      </c>
+      <c r="D6" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(how fast?)</t>
+        </is>
+      </c>
+      <c r="E6" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(which template?)</t>
+        </is>
+      </c>
+      <c r="F6" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(which tools?)</t>
+        </is>
+      </c>
+      <c r="G6" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(what's produced?)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="22" t="inlineStr">
         <is>
           <t>6. Resolution</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="22" t="inlineStr">
         <is>
           <t>Implement fix; deploy changes; validate in staging then production</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Engineering Team / DevOps</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>Depends on fix</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>Resolution Implementation Plan</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>GitHub, CI/CD Pipeline</t>
-        </is>
-      </c>
-      <c r="G7" s="7" t="inlineStr">
-        <is>
-          <t>Fix deployed and verified</t>
+      <c r="C7" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(who owns this step?)</t>
+        </is>
+      </c>
+      <c r="D7" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(how fast?)</t>
+        </is>
+      </c>
+      <c r="E7" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(which template?)</t>
+        </is>
+      </c>
+      <c r="F7" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(which tools?)</t>
+        </is>
+      </c>
+      <c r="G7" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(what's produced?)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="22" t="inlineStr">
         <is>
           <t>7. Verification</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>Confirm resolution effectiveness; monitor metrics; user acceptance</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>QA / Product / Engineering</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>1-4 hours post-deploy</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>Verification Checklist</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>Monitoring dashboards, Tests</t>
-        </is>
-      </c>
-      <c r="G8" s="7" t="inlineStr">
-        <is>
-          <t>Resolution verified</t>
+      <c r="C8" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(who owns this step?)</t>
+        </is>
+      </c>
+      <c r="D8" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(how fast?)</t>
+        </is>
+      </c>
+      <c r="E8" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(which template?)</t>
+        </is>
+      </c>
+      <c r="F8" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(which tools?)</t>
+        </is>
+      </c>
+      <c r="G8" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(what's produced?)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="22" t="inlineStr">
         <is>
           <t>8. Customer Communication</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="22" t="inlineStr">
         <is>
           <t>Notify customers; provide status updates; explain impact</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>Product / Communications</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>Communication Templates</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>Email, Status Page, Social Media</t>
-        </is>
-      </c>
-      <c r="G9" s="7" t="inlineStr">
-        <is>
-          <t>Customers informed</t>
+      <c r="C9" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(who owns this step?)</t>
+        </is>
+      </c>
+      <c r="D9" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(how fast?)</t>
+        </is>
+      </c>
+      <c r="E9" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(which template?)</t>
+        </is>
+      </c>
+      <c r="F9" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(which tools?)</t>
+        </is>
+      </c>
+      <c r="G9" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(what's produced?)</t>
         </is>
       </c>
     </row>
     <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="14" t="inlineStr">
-        <is>
-          <t>6. Resolution</t>
-        </is>
-      </c>
-      <c r="B10" s="14" t="inlineStr">
-        <is>
-          <t>Implement fix; deploy changes; validate in staging then production</t>
-        </is>
-      </c>
-      <c r="C10" s="14" t="inlineStr">
-        <is>
-          <t>Engineering Team / DevOps</t>
-        </is>
-      </c>
-      <c r="D10" s="14" t="inlineStr">
-        <is>
-          <t>Depends on fix</t>
-        </is>
-      </c>
-      <c r="E10" s="15" t="n"/>
-      <c r="F10" s="15" t="n"/>
-      <c r="G10" s="14" t="inlineStr">
-        <is>
-          <t>Fix deployed and verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A10" s="22" t="inlineStr">
         <is>
           <t>9. Post-Incident Review</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B10" s="22" t="inlineStr">
         <is>
           <t>"Conduct blameless postmortem meeting; document lessons learned; identify systemic improvements"
 Reasoning: Blameless approach encourages honest analysis; systematic documentation ensures findings are actionable; this step transforms incident experience into organizational learning.</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
-        <is>
-          <t>"Incident Commander, Engineering Lead, affected team members, Product Manager, Data Science Lead"
-Reasoning: Incident Commander ensures process integrity; Engineering/Data Science provide technical insights; Product understands customer impact; diverse perspectives identify root causes.</t>
-        </is>
-      </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>"Within 48 hours of incident resolution"
-Reasoning: Quick turnaround captures fresh memory and emotional context; within 48 hours ensures urgency without fatigue; too late and details are forgotten.</t>
-        </is>
-      </c>
-      <c r="E11" s="13" t="inlineStr">
-        <is>
-          <t>"Postmortem document with timeline, root cause, contributing factors, action items with owners and deadlines"
-Reasoning: Structured documentation ensures completeness; clear ownership and deadlines drive accountability; shared document enables transparency and organizational learning.</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>Zoom, Confluence, Jira</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="C10" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(who owns this step?)</t>
+        </is>
+      </c>
+      <c r="D10" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(how fast?)</t>
+        </is>
+      </c>
+      <c r="E10" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(which template?)</t>
+        </is>
+      </c>
+      <c r="F10" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(which tools?)</t>
+        </is>
+      </c>
+      <c r="G10" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(what's produced?)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="22" t="inlineStr">
         <is>
           <t>10. Knowledge Base Update</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B11" s="22" t="inlineStr">
         <is>
           <t>"Update runbooks with new procedures; add incident patterns to knowledge base; document root causes and solutions; update monitoring thresholds"
 Reasoning: Runbook updates improve response for similar future incidents; knowledge base prevents rediscovery; monitoring improvements provide earlier detection.</t>
         </is>
       </c>
-      <c r="C12" s="13" t="inlineStr">
-        <is>
-          <t>"Knowledge Manager, Technical Writer, and relevant technical teams who handled the incident"
-Reasoning: Knowledge Manager ensures quality and consistency; Technical Writers ensure clarity for future teams; involved technical teams capture accurate details.</t>
-        </is>
-      </c>
-      <c r="D12" s="13" t="inlineStr">
-        <is>
-          <t>"Within 5 business days of incident resolution"
-Reasoning: 5-day window allows action items to be completed before documentation; reasonable timeline avoids documentation backlog; ensures knowledge is current.</t>
-        </is>
-      </c>
-      <c r="E12" s="13" t="inlineStr">
-        <is>
-          <t>"Updated runbooks in Confluence, new alerting rules in monitoring system, root cause article in knowledge base"
-Reasoning: Confluence ensures team can find procedures; updated alerts prevent recurrence; knowledge base article enables transfer of learning across organization.</t>
-        </is>
-      </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>Confluence, GitHub Wiki</t>
+      <c r="C11" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(who owns this step?)</t>
+        </is>
+      </c>
+      <c r="D11" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(how fast?)</t>
+        </is>
+      </c>
+      <c r="E11" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(which template?)</t>
+        </is>
+      </c>
+      <c r="F11" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(which tools?)</t>
+        </is>
+      </c>
+      <c r="G11" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(what's produced?)</t>
         </is>
       </c>
     </row>
@@ -2041,7 +2154,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -2079,270 +2192,268 @@
       </c>
     </row>
     <row r="2" ht="40" customHeight="1">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="22" t="inlineStr">
         <is>
           <t>Incident Timeline</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="B2" s="22" t="inlineStr">
         <is>
           <t>Document all events chronologically from detection to resolution</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" s="22" t="inlineStr">
         <is>
           <t>When detected? Who notified? When were teams engaged? Key milestones?</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="D2" s="22" t="inlineStr">
         <is>
           <t>Incident Commander</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="E2" s="22" t="inlineStr">
         <is>
           <t>1 day post-incident</t>
         </is>
       </c>
     </row>
     <row r="3" ht="40" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="22" t="inlineStr">
         <is>
           <t>Root Cause Analysis</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="22" t="inlineStr">
         <is>
           <t>Investigate underlying causes; focus on systemic issues, not blame</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="22" t="inlineStr">
         <is>
           <t>Primary cause? Contributing factors? How was issue introduced? Prevention?</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="22" t="inlineStr">
         <is>
           <t>Technical Lead</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="22" t="inlineStr">
         <is>
           <t>3 days post-incident</t>
         </is>
       </c>
     </row>
     <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>Impact Assessment</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="22" t="inlineStr">
         <is>
           <t>Quantify actual impact on users, systems, and business metrics</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>Users affected? Duration? Business cost? Reputational impact?</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>Product / Analytics</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>2 days post-incident</t>
+      <c r="C4" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(what questions matter here?)</t>
+        </is>
+      </c>
+      <c r="D4" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(who owns this?)</t>
+        </is>
+      </c>
+      <c r="E4" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(by when?)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>Response Effectiveness</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>Evaluate how well response procedures and teams performed</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Were runbooks adequate? Team response speed? Communication quality?</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>Incident Manager</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>2 days post-incident</t>
+      <c r="C5" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(what questions matter here?)</t>
+        </is>
+      </c>
+      <c r="D5" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(who owns this?)</t>
+        </is>
+      </c>
+      <c r="E5" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(by when?)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>Lessons Learned</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
         <is>
           <t>Identify what went well and what could be improved</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>What went well? What to improve? What surprised us? Key insights?</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>All Team Members</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>3 days post-incident</t>
+      <c r="C6" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(what questions matter here?)</t>
+        </is>
+      </c>
+      <c r="D6" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(who owns this?)</t>
+        </is>
+      </c>
+      <c r="E6" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(by when?)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="22" t="inlineStr">
         <is>
           <t>Preventive Measures</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="22" t="inlineStr">
         <is>
           <t>Recommend specific changes to prevent recurrence</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>How to prevent this? Monitoring gaps? Process improvements?</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>Technical Leads</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>5 days post-incident</t>
+      <c r="C7" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(what questions matter here?)</t>
+        </is>
+      </c>
+      <c r="D7" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(who owns this?)</t>
+        </is>
+      </c>
+      <c r="E7" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(by when?)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="14" t="inlineStr">
-        <is>
-          <t>Preventive Measures</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="inlineStr">
-        <is>
-          <t>Recommend specific changes to prevent recurrence</t>
-        </is>
-      </c>
-      <c r="C8" s="14" t="inlineStr">
-        <is>
-          <t>How to prevent this? Monitoring gaps? Process improvements?</t>
-        </is>
-      </c>
-      <c r="D8" s="15" t="n"/>
-      <c r="E8" s="15" t="n"/>
+      <c r="A8" s="22" t="inlineStr">
+        <is>
+          <t>Action Items</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>List specific improvements with ownership and deadlines</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(what questions matter here?)</t>
+        </is>
+      </c>
+      <c r="D8" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(who owns this?)</t>
+        </is>
+      </c>
+      <c r="E8" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(by when?)</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>Action Items</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>List specific improvements with ownership and deadlines</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>What changes? Who owns each? Deadlines? How to track completion?</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>Project Manager</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>5 days post-incident</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A9" s="22" t="inlineStr">
         <is>
           <t>Communication Effectiveness</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B9" s="22" t="inlineStr">
         <is>
           <t>"Evaluate timeliness, accuracy, and clarity of customer and stakeholder communications throughout incident lifecycle"
 Reasoning: Timeliness assessment shows if notifications met SLAs; accuracy review catches misleading information; clarity ensures diverse audiences understood impact.</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
-        <is>
-          <t>"Were stakeholders informed within communication SLAs? Was information accurate and complete? Did tone match incident severity? Were updates consistent across channels?"
-Reasoning: SLA assessment ensures process compliance; accuracy prevents loss of trust; tone alignment demonstrates professional judgment; consistency prevents confusion.</t>
-        </is>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>"Communications Lead / Customer Relations Director"
-Reasoning: Communications team is accountable for message delivery; they understand audience expectations; they can improve templates and procedures.</t>
-        </is>
-      </c>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>2 days post-incident</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="C9" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(what questions matter here?)</t>
+        </is>
+      </c>
+      <c r="D9" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(who owns this?)</t>
+        </is>
+      </c>
+      <c r="E9" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(by when?)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="40" customHeight="1">
+      <c r="A10" s="22" t="inlineStr">
         <is>
           <t>Follow-up Schedule</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B10" s="22" t="inlineStr">
         <is>
           <t>"Establish schedule to verify completion of action items and monitor for incident recurrence"
 Reasoning: Scheduled follow-up ensures accountability; verification prevents items from slipping; monitoring catches early signs of recurrence.</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
-        <is>
-          <t>"When will action items be reviewed? What completion criteria define success? How will we verify the fix works in production? What metrics indicate recurrence?"
-Reasoning: Review schedule enforces deadlines; completion criteria ensure quality; production verification prevents regression; metrics provide early warning.</t>
-        </is>
-      </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>"Project Manager / Incident Commander"
-Reasoning: Project Manager tracks deliverables; Incident Commander ensures organizational learning; both are accountable for closure.</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>7 days post-incident</t>
+      <c r="C10" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(what questions matter here?)</t>
+        </is>
+      </c>
+      <c r="D10" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(who owns this?)</t>
+        </is>
+      </c>
+      <c r="E10" s="23" t="inlineStr">
+        <is>
+          <t>TO BE FILLED
+(by when?)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
L9: correct over-blanking — restore Reporting Workflow + Post-Incident Review to original
Previous commit over-blanked all four incident sheets by copying the whole
project-repo fix. Only Incident Playbook and Severity Classification were
genuinely identical to the solution; those stay blanked. Reporting Workflow and
Post-Incident Review were already proper exercises (matching the classroom
description) and are now restored to their original state.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lesson-9-ai-incident-management/exercises/starter/incident_response_starter.xlsx
+++ b/lesson-9-ai-incident-management/exercises/starter/incident_response_starter.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -54,10 +54,6 @@
       <i val="1"/>
       <color rgb="FF888888"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="FF888888"/>
     </font>
   </fonts>
   <fills count="14">
@@ -129,12 +125,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4EC"/>
+        <fgColor rgb="00D6E4F0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D6E4F0"/>
+        <fgColor rgb="00FCE4EC"/>
       </patternFill>
     </fill>
   </fills>
@@ -156,7 +152,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -199,20 +195,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -580,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -712,37 +698,6 @@
       <c r="A17" s="5" t="inlineStr">
         <is>
           <t>• Must report certain incidents to NTSB and FTA within mandated timeframes</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="16" t="inlineStr">
-        <is>
-          <t>COLOR LEGEND:</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="17" t="inlineStr">
-        <is>
-          <t>Pre-filled</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Context provided — do not change.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="18" t="inlineStr">
-        <is>
-          <t>Your work</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Cells marked TO BE FILLED — replace with your answer. Gray hints are prompts, not answers.</t>
         </is>
       </c>
     </row>
@@ -862,37 +817,37 @@
           <t>Routes through certain neighborhoods receive longer travel times</t>
         </is>
       </c>
-      <c r="E2" s="22" t="inlineStr">
+      <c r="E2" s="16" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
       </c>
-      <c r="F2" s="22" t="inlineStr">
+      <c r="F2" s="16" t="inlineStr">
         <is>
           <t>Monitor route fairness metrics across regions; compare avg travel times</t>
         </is>
       </c>
-      <c r="G2" s="22" t="inlineStr">
+      <c r="G2" s="16" t="inlineStr">
         <is>
           <t>Pause affected routes; escalate to ML team; notify operations</t>
         </is>
       </c>
-      <c r="H2" s="22" t="inlineStr">
+      <c r="H2" s="16" t="inlineStr">
         <is>
           <t>Review training data distribution; analyze prediction patterns by geography</t>
         </is>
       </c>
-      <c r="I2" s="22" t="inlineStr">
+      <c r="I2" s="16" t="inlineStr">
         <is>
           <t>Retrain with balanced data; implement fairness constraints; add monitoring</t>
         </is>
       </c>
-      <c r="J2" s="22" t="inlineStr">
+      <c r="J2" s="16" t="inlineStr">
         <is>
           <t>Notify affected route managers; customer support alert</t>
         </is>
       </c>
-      <c r="K2" s="22" t="inlineStr">
+      <c r="K2" s="16" t="inlineStr">
         <is>
           <t>Document root cause; update training pipeline; implement fairness dashboard</t>
         </is>
@@ -919,37 +874,37 @@
           <t>Chatbot provides rude or discriminatory responses to passenger inquiries</t>
         </is>
       </c>
-      <c r="E3" s="22" t="inlineStr">
+      <c r="E3" s="16" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
       </c>
-      <c r="F3" s="22" t="inlineStr">
+      <c r="F3" s="16" t="inlineStr">
         <is>
           <t>Content filtering; customer complaints; automated toxicity detection</t>
         </is>
       </c>
-      <c r="G3" s="22" t="inlineStr">
+      <c r="G3" s="16" t="inlineStr">
         <is>
           <t>Disable chatbot; escalate to content team; begin log analysis</t>
         </is>
       </c>
-      <c r="H3" s="22" t="inlineStr">
+      <c r="H3" s="16" t="inlineStr">
         <is>
           <t>Review chat logs; identify trigger phrases; check outputs for toxicity</t>
         </is>
       </c>
-      <c r="I3" s="22" t="inlineStr">
+      <c r="I3" s="16" t="inlineStr">
         <is>
           <t>Apply content filters; retrain with safer examples; add guardrails</t>
         </is>
       </c>
-      <c r="J3" s="22" t="inlineStr">
+      <c r="J3" s="16" t="inlineStr">
         <is>
           <t>Apologize to passengers; notify customer service teams</t>
         </is>
       </c>
-      <c r="K3" s="22" t="inlineStr">
+      <c r="K3" s="16" t="inlineStr">
         <is>
           <t>Update chatbot guidelines; implement content moderation</t>
         </is>
@@ -976,41 +931,41 @@
           <t>Route accuracy drops from 94% to 78% during morning rush</t>
         </is>
       </c>
-      <c r="E4" s="19" t="inlineStr">
+      <c r="E4" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (which severity? S1–S4)</t>
         </is>
       </c>
-      <c r="F4" s="19" t="inlineStr">
+      <c r="F4" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (how would you catch it?)</t>
         </is>
       </c>
-      <c r="G4" s="19" t="inlineStr">
+      <c r="G4" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (first-hour containment?)</t>
         </is>
       </c>
-      <c r="H4" s="19" t="inlineStr">
+      <c r="H4" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED</t>
         </is>
       </c>
-      <c r="I4" s="19" t="inlineStr">
+      <c r="I4" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED</t>
         </is>
       </c>
-      <c r="J4" s="19" t="inlineStr">
+      <c r="J4" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (who needs to know?)</t>
         </is>
       </c>
-      <c r="K4" s="19" t="inlineStr">
+      <c r="K4" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (prevent recurrence?)</t>
@@ -1038,41 +993,41 @@
           <t>Personal location data and payment info exposed via API vulnerability</t>
         </is>
       </c>
-      <c r="E5" s="19" t="inlineStr">
+      <c r="E5" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (which severity? S1–S4)</t>
         </is>
       </c>
-      <c r="F5" s="19" t="inlineStr">
+      <c r="F5" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (how would you catch it?)</t>
         </is>
       </c>
-      <c r="G5" s="19" t="inlineStr">
+      <c r="G5" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (first-hour containment?)</t>
         </is>
       </c>
-      <c r="H5" s="19" t="inlineStr">
+      <c r="H5" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED</t>
         </is>
       </c>
-      <c r="I5" s="19" t="inlineStr">
+      <c r="I5" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED</t>
         </is>
       </c>
-      <c r="J5" s="19" t="inlineStr">
+      <c r="J5" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (who needs to know?)</t>
         </is>
       </c>
-      <c r="K5" s="19" t="inlineStr">
+      <c r="K5" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (prevent recurrence?)</t>
@@ -1100,41 +1055,41 @@
           <t>Route guidance includes non-existent roads or omits safety warnings</t>
         </is>
       </c>
-      <c r="E6" s="19" t="inlineStr">
+      <c r="E6" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (which severity? S1–S4)</t>
         </is>
       </c>
-      <c r="F6" s="19" t="inlineStr">
+      <c r="F6" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (how would you catch it?)</t>
         </is>
       </c>
-      <c r="G6" s="19" t="inlineStr">
+      <c r="G6" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (first-hour containment?)</t>
         </is>
       </c>
-      <c r="H6" s="19" t="inlineStr">
+      <c r="H6" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED</t>
         </is>
       </c>
-      <c r="I6" s="19" t="inlineStr">
+      <c r="I6" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED</t>
         </is>
       </c>
-      <c r="J6" s="19" t="inlineStr">
+      <c r="J6" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (who needs to know?)</t>
         </is>
       </c>
-      <c r="K6" s="19" t="inlineStr">
+      <c r="K6" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (prevent recurrence?)</t>
@@ -1162,41 +1117,41 @@
           <t>Kubernetes cluster crash; database connection failure</t>
         </is>
       </c>
-      <c r="E7" s="19" t="inlineStr">
+      <c r="E7" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (which severity? S1–S4)</t>
         </is>
       </c>
-      <c r="F7" s="19" t="inlineStr">
+      <c r="F7" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (how would you catch it?)</t>
         </is>
       </c>
-      <c r="G7" s="19" t="inlineStr">
+      <c r="G7" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (first-hour containment?)</t>
         </is>
       </c>
-      <c r="H7" s="19" t="inlineStr">
+      <c r="H7" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED</t>
         </is>
       </c>
-      <c r="I7" s="19" t="inlineStr">
+      <c r="I7" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED</t>
         </is>
       </c>
-      <c r="J7" s="19" t="inlineStr">
+      <c r="J7" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (who needs to know?)</t>
         </is>
       </c>
-      <c r="K7" s="19" t="inlineStr">
+      <c r="K7" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (prevent recurrence?)</t>
@@ -1224,41 +1179,41 @@
           <t>Decisions made without explainability; violates data residency requirements</t>
         </is>
       </c>
-      <c r="E8" s="19" t="inlineStr">
+      <c r="E8" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (which severity? S1–S4)</t>
         </is>
       </c>
-      <c r="F8" s="19" t="inlineStr">
+      <c r="F8" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (how would you catch it?)</t>
         </is>
       </c>
-      <c r="G8" s="19" t="inlineStr">
+      <c r="G8" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (first-hour containment?)</t>
         </is>
       </c>
-      <c r="H8" s="19" t="inlineStr">
+      <c r="H8" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED</t>
         </is>
       </c>
-      <c r="I8" s="19" t="inlineStr">
+      <c r="I8" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED</t>
         </is>
       </c>
-      <c r="J8" s="19" t="inlineStr">
+      <c r="J8" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (who needs to know?)</t>
         </is>
       </c>
-      <c r="K8" s="19" t="inlineStr">
+      <c r="K8" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (prevent recurrence?)</t>
@@ -1286,41 +1241,41 @@
           <t>Coordinated requests with malicious patterns designed to degrade service</t>
         </is>
       </c>
-      <c r="E9" s="19" t="inlineStr">
+      <c r="E9" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (which severity? S1–S4)</t>
         </is>
       </c>
-      <c r="F9" s="19" t="inlineStr">
+      <c r="F9" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (how would you catch it?)</t>
         </is>
       </c>
-      <c r="G9" s="19" t="inlineStr">
+      <c r="G9" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (first-hour containment?)</t>
         </is>
       </c>
-      <c r="H9" s="19" t="inlineStr">
+      <c r="H9" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED</t>
         </is>
       </c>
-      <c r="I9" s="19" t="inlineStr">
+      <c r="I9" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED</t>
         </is>
       </c>
-      <c r="J9" s="19" t="inlineStr">
+      <c r="J9" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (who needs to know?)</t>
         </is>
       </c>
-      <c r="K9" s="19" t="inlineStr">
+      <c r="K9" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (prevent recurrence?)</t>
@@ -1348,41 +1303,41 @@
           <t>Historical route data tampered with to introduce systematic bias</t>
         </is>
       </c>
-      <c r="E10" s="19" t="inlineStr">
+      <c r="E10" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (which severity? S1–S4)</t>
         </is>
       </c>
-      <c r="F10" s="19" t="inlineStr">
+      <c r="F10" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (how would you catch it?)</t>
         </is>
       </c>
-      <c r="G10" s="19" t="inlineStr">
+      <c r="G10" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (first-hour containment?)</t>
         </is>
       </c>
-      <c r="H10" s="19" t="inlineStr">
+      <c r="H10" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED</t>
         </is>
       </c>
-      <c r="I10" s="19" t="inlineStr">
+      <c r="I10" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED</t>
         </is>
       </c>
-      <c r="J10" s="19" t="inlineStr">
+      <c r="J10" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (who needs to know?)</t>
         </is>
       </c>
-      <c r="K10" s="19" t="inlineStr">
+      <c r="K10" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (prevent recurrence?)</t>
@@ -1410,41 +1365,41 @@
           <t>Former contractor retains access; API key exposed in public repository</t>
         </is>
       </c>
-      <c r="E11" s="19" t="inlineStr">
+      <c r="E11" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (which severity? S1–S4)</t>
         </is>
       </c>
-      <c r="F11" s="19" t="inlineStr">
+      <c r="F11" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (how would you catch it?)</t>
         </is>
       </c>
-      <c r="G11" s="19" t="inlineStr">
+      <c r="G11" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (first-hour containment?)</t>
         </is>
       </c>
-      <c r="H11" s="19" t="inlineStr">
+      <c r="H11" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED</t>
         </is>
       </c>
-      <c r="I11" s="19" t="inlineStr">
+      <c r="I11" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED</t>
         </is>
       </c>
-      <c r="J11" s="19" t="inlineStr">
+      <c r="J11" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (who needs to know?)</t>
         </is>
       </c>
-      <c r="K11" s="19" t="inlineStr">
+      <c r="K11" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (prevent recurrence?)</t>
@@ -1522,27 +1477,27 @@
           <t>S1</t>
         </is>
       </c>
-      <c r="C2" s="22" t="inlineStr">
+      <c r="C2" s="16" t="inlineStr">
         <is>
           <t>Immediate safety risk; potential data breach; system unavailable; passenger safety compromised</t>
         </is>
       </c>
-      <c r="D2" s="22" t="inlineStr">
+      <c r="D2" s="16" t="inlineStr">
         <is>
           <t>&lt; 15 minutes</t>
         </is>
       </c>
-      <c r="E2" s="22" t="inlineStr">
+      <c r="E2" s="16" t="inlineStr">
         <is>
           <t>CEO/Board; Legal; Chief Security Officer; NTSB/FTA</t>
         </is>
       </c>
-      <c r="F2" s="22" t="inlineStr">
+      <c r="F2" s="16" t="inlineStr">
         <is>
           <t>All stakeholders; customers; regulators; media</t>
         </is>
       </c>
-      <c r="G2" s="22" t="inlineStr">
+      <c r="G2" s="16" t="inlineStr">
         <is>
           <t>Data breach; System outage; Safety-critical hallucination</t>
         </is>
@@ -1559,30 +1514,30 @@
           <t>S2</t>
         </is>
       </c>
-      <c r="C3" s="19" t="inlineStr">
+      <c r="C3" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (harm to whom?)</t>
         </is>
       </c>
-      <c r="D3" s="19" t="inlineStr">
+      <c r="D3" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (how fast?)</t>
         </is>
       </c>
-      <c r="E3" s="19" t="inlineStr">
+      <c r="E3" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (escalate to whom?)</t>
         </is>
       </c>
-      <c r="F3" s="19" t="inlineStr">
+      <c r="F3" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED</t>
         </is>
       </c>
-      <c r="G3" s="19" t="inlineStr">
+      <c r="G3" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (which incidents fit?)</t>
@@ -1600,30 +1555,30 @@
           <t>S3</t>
         </is>
       </c>
-      <c r="C4" s="19" t="inlineStr">
+      <c r="C4" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (harm to whom?)</t>
         </is>
       </c>
-      <c r="D4" s="19" t="inlineStr">
+      <c r="D4" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (how fast?)</t>
         </is>
       </c>
-      <c r="E4" s="19" t="inlineStr">
+      <c r="E4" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (escalate to whom?)</t>
         </is>
       </c>
-      <c r="F4" s="19" t="inlineStr">
+      <c r="F4" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED</t>
         </is>
       </c>
-      <c r="G4" s="19" t="inlineStr">
+      <c r="G4" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (which incidents fit?)</t>
@@ -1641,30 +1596,30 @@
           <t>S4</t>
         </is>
       </c>
-      <c r="C5" s="19" t="inlineStr">
+      <c r="C5" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (harm to whom?)</t>
         </is>
       </c>
-      <c r="D5" s="19" t="inlineStr">
+      <c r="D5" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (how fast?)</t>
         </is>
       </c>
-      <c r="E5" s="19" t="inlineStr">
+      <c r="E5" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (escalate to whom?)</t>
         </is>
       </c>
-      <c r="F5" s="19" t="inlineStr">
+      <c r="F5" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED</t>
         </is>
       </c>
-      <c r="G5" s="19" t="inlineStr">
+      <c r="G5" s="17" t="inlineStr">
         <is>
           <t>TO BE FILLED
 (which incidents fit?)</t>
@@ -1682,7 +1637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1732,414 +1687,399 @@
       </c>
     </row>
     <row r="2" ht="40" customHeight="1">
-      <c r="A2" s="22" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>1. Detection</t>
         </is>
       </c>
-      <c r="B2" s="22" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>Identify anomaly through monitoring, alerts, or user reports</t>
         </is>
       </c>
-      <c r="C2" s="22" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>Monitoring System / Operations Team</t>
         </is>
       </c>
-      <c r="D2" s="22" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>Real-time to 5 min</t>
         </is>
       </c>
-      <c r="E2" s="22" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>Incident Alert Template</t>
         </is>
       </c>
-      <c r="F2" s="22" t="inlineStr">
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>Prometheus, DataDog, Support System</t>
         </is>
       </c>
-      <c r="G2" s="22" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>Incident ticket created</t>
         </is>
       </c>
     </row>
     <row r="3" ht="40" customHeight="1">
-      <c r="A3" s="22" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>2. Triage</t>
         </is>
       </c>
-      <c r="B3" s="22" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>Verify incident; assess immediate impact; gather initial context</t>
         </is>
       </c>
-      <c r="C3" s="22" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>On-Call Engineer / Incident Manager</t>
         </is>
       </c>
-      <c r="D3" s="22" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>5-15 minutes</t>
         </is>
       </c>
-      <c r="E3" s="22" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>Triage Assessment Form</t>
         </is>
       </c>
-      <c r="F3" s="22" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>PagerDuty, Jira</t>
         </is>
       </c>
-      <c r="G3" s="22" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>Confirmed incident with initial severity</t>
         </is>
       </c>
     </row>
     <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="22" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>3. Classification</t>
         </is>
       </c>
-      <c r="B4" s="22" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Determine severity; assign category; set SLA response time</t>
         </is>
       </c>
-      <c r="C4" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(who owns this step?)</t>
-        </is>
-      </c>
-      <c r="D4" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(how fast?)</t>
-        </is>
-      </c>
-      <c r="E4" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(which template?)</t>
-        </is>
-      </c>
-      <c r="F4" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(which tools?)</t>
-        </is>
-      </c>
-      <c r="G4" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(what's produced?)</t>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Incident Manager / Tech Lead</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>10-20 minutes</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Classification Matrix</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Incident Management Tool, Slack</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>Incident classified with severity and SLA</t>
         </is>
       </c>
     </row>
     <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="22" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>4. Initial Response</t>
         </is>
       </c>
-      <c r="B5" s="22" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Execute containment actions per playbook; engage necessary teams</t>
         </is>
       </c>
-      <c r="C5" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(who owns this step?)</t>
-        </is>
-      </c>
-      <c r="D5" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(how fast?)</t>
-        </is>
-      </c>
-      <c r="E5" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(which template?)</t>
-        </is>
-      </c>
-      <c r="F5" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(which tools?)</t>
-        </is>
-      </c>
-      <c r="G5" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(what's produced?)</t>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Engineering Lead / Operations</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Within SLA</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Incident Response Checklist</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Runbooks, Slack, War Room</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Incident contained; teams engaged</t>
         </is>
       </c>
     </row>
     <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>5. Investigation</t>
         </is>
       </c>
-      <c r="B6" s="22" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Detailed analysis; gather logs and metrics; identify root cause</t>
         </is>
       </c>
-      <c r="C6" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(who owns this step?)</t>
-        </is>
-      </c>
-      <c r="D6" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(how fast?)</t>
-        </is>
-      </c>
-      <c r="E6" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(which template?)</t>
-        </is>
-      </c>
-      <c r="F6" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(which tools?)</t>
-        </is>
-      </c>
-      <c r="G6" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(what's produced?)</t>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Data Scientists / Engineers / Security</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>1-48 hours</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Investigation Log Template</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>ELK Stack, Jupyter, Git</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>Root cause identified</t>
         </is>
       </c>
     </row>
     <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="22" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>6. Resolution</t>
         </is>
       </c>
-      <c r="B7" s="22" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Implement fix; deploy changes; validate in staging then production</t>
         </is>
       </c>
-      <c r="C7" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(who owns this step?)</t>
-        </is>
-      </c>
-      <c r="D7" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(how fast?)</t>
-        </is>
-      </c>
-      <c r="E7" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(which template?)</t>
-        </is>
-      </c>
-      <c r="F7" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(which tools?)</t>
-        </is>
-      </c>
-      <c r="G7" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(what's produced?)</t>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Engineering Team / DevOps</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Depends on fix</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Resolution Implementation Plan</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>GitHub, CI/CD Pipeline</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Fix deployed and verified</t>
         </is>
       </c>
     </row>
     <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>7. Verification</t>
         </is>
       </c>
-      <c r="B8" s="22" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Confirm resolution effectiveness; monitor metrics; user acceptance</t>
         </is>
       </c>
-      <c r="C8" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(who owns this step?)</t>
-        </is>
-      </c>
-      <c r="D8" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(how fast?)</t>
-        </is>
-      </c>
-      <c r="E8" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(which template?)</t>
-        </is>
-      </c>
-      <c r="F8" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(which tools?)</t>
-        </is>
-      </c>
-      <c r="G8" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(what's produced?)</t>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>QA / Product / Engineering</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>1-4 hours post-deploy</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Verification Checklist</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Monitoring dashboards, Tests</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>Resolution verified</t>
         </is>
       </c>
     </row>
     <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="22" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>8. Customer Communication</t>
         </is>
       </c>
-      <c r="B9" s="22" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>Notify customers; provide status updates; explain impact</t>
         </is>
       </c>
-      <c r="C9" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(who owns this step?)</t>
-        </is>
-      </c>
-      <c r="D9" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(how fast?)</t>
-        </is>
-      </c>
-      <c r="E9" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(which template?)</t>
-        </is>
-      </c>
-      <c r="F9" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(which tools?)</t>
-        </is>
-      </c>
-      <c r="G9" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(what's produced?)</t>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Product / Communications</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Communication Templates</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>Email, Status Page, Social Media</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>Customers informed</t>
         </is>
       </c>
     </row>
     <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="22" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>6. Resolution</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>Implement fix; deploy changes; validate in staging then production</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>Engineering Team / DevOps</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>Depends on fix</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="n"/>
+      <c r="F10" s="15" t="n"/>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>Fix deployed and verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>9. Post-Incident Review</t>
         </is>
       </c>
-      <c r="B10" s="22" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>"Conduct blameless postmortem meeting; document lessons learned; identify systemic improvements"
 Reasoning: Blameless approach encourages honest analysis; systematic documentation ensures findings are actionable; this step transforms incident experience into organizational learning.</t>
         </is>
       </c>
-      <c r="C10" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(who owns this step?)</t>
-        </is>
-      </c>
-      <c r="D10" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(how fast?)</t>
-        </is>
-      </c>
-      <c r="E10" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(which template?)</t>
-        </is>
-      </c>
-      <c r="F10" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(which tools?)</t>
-        </is>
-      </c>
-      <c r="G10" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(what's produced?)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="22" t="inlineStr">
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>"Incident Commander, Engineering Lead, affected team members, Product Manager, Data Science Lead"
+Reasoning: Incident Commander ensures process integrity; Engineering/Data Science provide technical insights; Product understands customer impact; diverse perspectives identify root causes.</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>"Within 48 hours of incident resolution"
+Reasoning: Quick turnaround captures fresh memory and emotional context; within 48 hours ensures urgency without fatigue; too late and details are forgotten.</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>"Postmortem document with timeline, root cause, contributing factors, action items with owners and deadlines"
+Reasoning: Structured documentation ensures completeness; clear ownership and deadlines drive accountability; shared document enables transparency and organizational learning.</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Zoom, Confluence, Jira</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>10. Knowledge Base Update</t>
         </is>
       </c>
-      <c r="B11" s="22" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>"Update runbooks with new procedures; add incident patterns to knowledge base; document root causes and solutions; update monitoring thresholds"
 Reasoning: Runbook updates improve response for similar future incidents; knowledge base prevents rediscovery; monitoring improvements provide earlier detection.</t>
         </is>
       </c>
-      <c r="C11" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(who owns this step?)</t>
-        </is>
-      </c>
-      <c r="D11" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(how fast?)</t>
-        </is>
-      </c>
-      <c r="E11" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(which template?)</t>
-        </is>
-      </c>
-      <c r="F11" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(which tools?)</t>
-        </is>
-      </c>
-      <c r="G11" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(what's produced?)</t>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>"Knowledge Manager, Technical Writer, and relevant technical teams who handled the incident"
+Reasoning: Knowledge Manager ensures quality and consistency; Technical Writers ensure clarity for future teams; involved technical teams capture accurate details.</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>"Within 5 business days of incident resolution"
+Reasoning: 5-day window allows action items to be completed before documentation; reasonable timeline avoids documentation backlog; ensures knowledge is current.</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>"Updated runbooks in Confluence, new alerting rules in monitoring system, root cause article in knowledge base"
+Reasoning: Confluence ensures team can find procedures; updated alerts prevent recurrence; knowledge base article enables transfer of learning across organization.</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>Confluence, GitHub Wiki</t>
         </is>
       </c>
     </row>
@@ -2154,7 +2094,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -2192,268 +2132,270 @@
       </c>
     </row>
     <row r="2" ht="40" customHeight="1">
-      <c r="A2" s="22" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>Incident Timeline</t>
         </is>
       </c>
-      <c r="B2" s="22" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>Document all events chronologically from detection to resolution</t>
         </is>
       </c>
-      <c r="C2" s="22" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>When detected? Who notified? When were teams engaged? Key milestones?</t>
         </is>
       </c>
-      <c r="D2" s="22" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>Incident Commander</t>
         </is>
       </c>
-      <c r="E2" s="22" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>1 day post-incident</t>
         </is>
       </c>
     </row>
     <row r="3" ht="40" customHeight="1">
-      <c r="A3" s="22" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Root Cause Analysis</t>
         </is>
       </c>
-      <c r="B3" s="22" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>Investigate underlying causes; focus on systemic issues, not blame</t>
         </is>
       </c>
-      <c r="C3" s="22" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>Primary cause? Contributing factors? How was issue introduced? Prevention?</t>
         </is>
       </c>
-      <c r="D3" s="22" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>Technical Lead</t>
         </is>
       </c>
-      <c r="E3" s="22" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>3 days post-incident</t>
         </is>
       </c>
     </row>
     <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="22" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Impact Assessment</t>
         </is>
       </c>
-      <c r="B4" s="22" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Quantify actual impact on users, systems, and business metrics</t>
         </is>
       </c>
-      <c r="C4" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(what questions matter here?)</t>
-        </is>
-      </c>
-      <c r="D4" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(who owns this?)</t>
-        </is>
-      </c>
-      <c r="E4" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(by when?)</t>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Users affected? Duration? Business cost? Reputational impact?</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Product / Analytics</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>2 days post-incident</t>
         </is>
       </c>
     </row>
     <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="22" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Response Effectiveness</t>
         </is>
       </c>
-      <c r="B5" s="22" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Evaluate how well response procedures and teams performed</t>
         </is>
       </c>
-      <c r="C5" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(what questions matter here?)</t>
-        </is>
-      </c>
-      <c r="D5" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(who owns this?)</t>
-        </is>
-      </c>
-      <c r="E5" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(by when?)</t>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Were runbooks adequate? Team response speed? Communication quality?</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Incident Manager</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>2 days post-incident</t>
         </is>
       </c>
     </row>
     <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Lessons Learned</t>
         </is>
       </c>
-      <c r="B6" s="22" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Identify what went well and what could be improved</t>
         </is>
       </c>
-      <c r="C6" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(what questions matter here?)</t>
-        </is>
-      </c>
-      <c r="D6" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(who owns this?)</t>
-        </is>
-      </c>
-      <c r="E6" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(by when?)</t>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>What went well? What to improve? What surprised us? Key insights?</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>All Team Members</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>3 days post-incident</t>
         </is>
       </c>
     </row>
     <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="22" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Preventive Measures</t>
         </is>
       </c>
-      <c r="B7" s="22" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Recommend specific changes to prevent recurrence</t>
         </is>
       </c>
-      <c r="C7" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(what questions matter here?)</t>
-        </is>
-      </c>
-      <c r="D7" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(who owns this?)</t>
-        </is>
-      </c>
-      <c r="E7" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(by when?)</t>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>How to prevent this? Monitoring gaps? Process improvements?</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Technical Leads</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>5 days post-incident</t>
         </is>
       </c>
     </row>
     <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>Preventive Measures</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>Recommend specific changes to prevent recurrence</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>How to prevent this? Monitoring gaps? Process improvements?</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="n"/>
+      <c r="E8" s="15" t="n"/>
+    </row>
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Action Items</t>
         </is>
       </c>
-      <c r="B8" s="22" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>List specific improvements with ownership and deadlines</t>
         </is>
       </c>
-      <c r="C8" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(what questions matter here?)</t>
-        </is>
-      </c>
-      <c r="D8" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(who owns this?)</t>
-        </is>
-      </c>
-      <c r="E8" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(by when?)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="22" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>What changes? Who owns each? Deadlines? How to track completion?</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Project Manager</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>5 days post-incident</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="40" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Communication Effectiveness</t>
         </is>
       </c>
-      <c r="B9" s="22" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>"Evaluate timeliness, accuracy, and clarity of customer and stakeholder communications throughout incident lifecycle"
 Reasoning: Timeliness assessment shows if notifications met SLAs; accuracy review catches misleading information; clarity ensures diverse audiences understood impact.</t>
         </is>
       </c>
-      <c r="C9" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(what questions matter here?)</t>
-        </is>
-      </c>
-      <c r="D9" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(who owns this?)</t>
-        </is>
-      </c>
-      <c r="E9" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(by when?)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="22" t="inlineStr">
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>"Were stakeholders informed within communication SLAs? Was information accurate and complete? Did tone match incident severity? Were updates consistent across channels?"
+Reasoning: SLA assessment ensures process compliance; accuracy prevents loss of trust; tone alignment demonstrates professional judgment; consistency prevents confusion.</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>"Communications Lead / Customer Relations Director"
+Reasoning: Communications team is accountable for message delivery; they understand audience expectations; they can improve templates and procedures.</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>2 days post-incident</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>Follow-up Schedule</t>
         </is>
       </c>
-      <c r="B10" s="22" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>"Establish schedule to verify completion of action items and monitor for incident recurrence"
 Reasoning: Scheduled follow-up ensures accountability; verification prevents items from slipping; monitoring catches early signs of recurrence.</t>
         </is>
       </c>
-      <c r="C10" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(what questions matter here?)</t>
-        </is>
-      </c>
-      <c r="D10" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(who owns this?)</t>
-        </is>
-      </c>
-      <c r="E10" s="23" t="inlineStr">
-        <is>
-          <t>TO BE FILLED
-(by when?)</t>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>"When will action items be reviewed? What completion criteria define success? How will we verify the fix works in production? What metrics indicate recurrence?"
+Reasoning: Review schedule enforces deadlines; completion criteria ensure quality; production verification prevents regression; metrics provide early warning.</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>"Project Manager / Incident Commander"
+Reasoning: Project Manager tracks deliverables; Incident Commander ensures organizational learning; both are accountable for closure.</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>7 days post-incident</t>
         </is>
       </c>
     </row>

</xml_diff>